<commit_message>
Regen outputs for newer pandas version
</commit_message>
<xml_diff>
--- a/tests/data/output/report_WithSplitBB.xlsx
+++ b/tests/data/output/report_WithSplitBB.xlsx
@@ -693,7 +693,7 @@
         <v>120</v>
       </c>
       <c r="O6" s="7">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="P6" s="6">
         <v>20</v>
@@ -705,7 +705,7 @@
         <v>100</v>
       </c>
       <c r="S6" s="7">
-        <v>20</v>
+        <v>20.0</v>
       </c>
       <c r="T6" s="6">
         <v>1</v>
@@ -740,7 +740,7 @@
         <v>120</v>
       </c>
       <c r="O7" s="7">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="P7" s="6">
         <v>20</v>
@@ -752,7 +752,7 @@
         <v>100</v>
       </c>
       <c r="S7" s="7">
-        <v>20</v>
+        <v>20.0</v>
       </c>
       <c r="T7" s="6">
         <v>1</v>
@@ -931,7 +931,7 @@
     </row>
     <row r="20" spans="1:1">
       <c r="A20" s="8">
-        <v>200</v>
+        <v>200.0</v>
       </c>
     </row>
     <row r="21" spans="1:1">
@@ -941,7 +941,7 @@
     </row>
     <row r="22" spans="1:1">
       <c r="A22" s="8">
-        <v>40</v>
+        <v>40.0</v>
       </c>
     </row>
     <row r="23" spans="1:1">

</xml_diff>